<commit_message>
realease: excel a pdf
</commit_message>
<xml_diff>
--- a/src/assets/docs/modeloGDR.xlsx
+++ b/src/assets/docs/modeloGDR.xlsx
@@ -581,7 +581,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="39">
+  <fonts count="38" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -618,12 +618,6 @@
     <font>
       <b/>
       <sz val="25"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="18"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -840,7 +834,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="16">
+  <fills count="15">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -856,12 +850,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FF012447"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FF037341"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -932,7 +920,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="37">
+  <borders count="35">
     <border>
       <left/>
       <right/>
@@ -1028,82 +1016,6 @@
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -1289,13 +1201,13 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
+      <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="medium">
+      <top style="thin">
         <color indexed="64"/>
       </top>
       <bottom/>
@@ -1305,59 +1217,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
       <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
         <color indexed="64"/>
       </right>
       <top/>
@@ -1372,30 +1232,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top/>
       <bottom style="thin">
         <color indexed="64"/>
       </bottom>
@@ -1410,488 +1246,595 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="153">
+  <cellXfs count="148">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="9" fontId="24" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="23" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="9" fontId="13" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="9" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="37" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="20" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="36" fillId="0" borderId="0" xfId="3" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="13" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="23" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="11" fillId="0" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="32" fillId="4" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="25" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="11" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="11" borderId="15" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="26" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="27" fillId="11" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection hidden="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="5" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="6" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="9" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="3" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="37" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="6" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="19" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <protection locked="0"/>
+    </xf>
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="20" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="21" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="22" fillId="13" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="21" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment vertical="center" wrapText="1"/>
       <protection hidden="1"/>
     </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="49" fontId="22" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="49" fontId="15" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="16" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="49" fontId="11" fillId="14" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="49" fontId="10" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="23" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="21" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="22" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="21" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="14" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="25" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="26" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="12" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="12" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="27" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="28" fillId="12" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection hidden="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="15" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="12" fillId="0" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="22" fillId="0" borderId="26" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="7" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="20" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="33" fillId="5" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="23" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="25" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="10" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="11" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="14" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="49" fontId="16" fillId="0" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="38" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="3" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="49" fontId="11" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="10" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="3"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="9" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-      <protection locked="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="35" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="4">
@@ -2053,8 +1996,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="77258" y="5349751"/>
-          <a:ext cx="530225" cy="488950"/>
+          <a:off x="77258" y="7290946"/>
+          <a:ext cx="543560" cy="488950"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2739,7 +2682,7 @@
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
   <dimension ref="B1:N46"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
     <col min="2" max="2" width="4.5546875" customWidth="1"/>
@@ -2757,7 +2700,7 @@
     <col min="15" max="26" width="11.44140625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:14" ht="12" customHeight="1" thickBot="1">
+    <row r="1" spans="2:14" ht="12" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
       <c r="D1" s="1"/>
@@ -2772,26 +2715,26 @@
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
     </row>
-    <row r="2" spans="2:14" ht="64.5" customHeight="1" thickBot="1">
-      <c r="B2" s="114" t="s">
+    <row r="2" spans="2:14" ht="64.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B2" s="41" t="s">
         <v>3</v>
       </c>
-      <c r="C2" s="115"/>
-      <c r="D2" s="115"/>
-      <c r="E2" s="115"/>
-      <c r="F2" s="115"/>
-      <c r="G2" s="115"/>
-      <c r="H2" s="115"/>
-      <c r="I2" s="115"/>
-      <c r="J2" s="115"/>
-      <c r="K2" s="115"/>
-      <c r="L2" s="116"/>
-      <c r="M2" s="117" t="s">
+      <c r="C2" s="133"/>
+      <c r="D2" s="133"/>
+      <c r="E2" s="133"/>
+      <c r="F2" s="133"/>
+      <c r="G2" s="133"/>
+      <c r="H2" s="133"/>
+      <c r="I2" s="133"/>
+      <c r="J2" s="133"/>
+      <c r="K2" s="133"/>
+      <c r="L2" s="134"/>
+      <c r="M2" s="42" t="s">
         <v>46</v>
       </c>
-      <c r="N2" s="118"/>
-    </row>
-    <row r="3" spans="2:14" ht="18.600000000000001" thickBot="1">
+      <c r="N2" s="132"/>
+    </row>
+    <row r="3" spans="2:14" ht="18.600000000000001" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B3" s="3"/>
       <c r="C3" s="4"/>
       <c r="D3" s="4"/>
@@ -2806,26 +2749,26 @@
       <c r="M3" s="4"/>
       <c r="N3" s="4"/>
     </row>
-    <row r="4" spans="2:14" ht="39.75" customHeight="1" thickBot="1">
-      <c r="B4" s="119" t="s">
+    <row r="4" spans="2:14" ht="39.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B4" s="130" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="120"/>
-      <c r="D4" s="121" t="s">
+      <c r="C4" s="131"/>
+      <c r="D4" s="127" t="s">
         <v>45</v>
       </c>
-      <c r="E4" s="121"/>
-      <c r="F4" s="121"/>
-      <c r="G4" s="121"/>
-      <c r="H4" s="121"/>
-      <c r="I4" s="121"/>
-      <c r="J4" s="121"/>
-      <c r="K4" s="121"/>
-      <c r="L4" s="121"/>
-      <c r="M4" s="121"/>
-      <c r="N4" s="122"/>
-    </row>
-    <row r="5" spans="2:14" ht="15" thickBot="1">
+      <c r="E4" s="128"/>
+      <c r="F4" s="128"/>
+      <c r="G4" s="128"/>
+      <c r="H4" s="128"/>
+      <c r="I4" s="128"/>
+      <c r="J4" s="128"/>
+      <c r="K4" s="128"/>
+      <c r="L4" s="128"/>
+      <c r="M4" s="128"/>
+      <c r="N4" s="129"/>
+    </row>
+    <row r="5" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B5" s="5"/>
       <c r="C5" s="6"/>
       <c r="D5" s="6"/>
@@ -2840,174 +2783,174 @@
       <c r="M5" s="6"/>
       <c r="N5" s="6"/>
     </row>
-    <row r="6" spans="2:14" ht="21.6" thickBot="1">
-      <c r="B6" s="123" t="s">
+    <row r="6" spans="2:14" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B6" s="110" t="s">
         <v>0</v>
       </c>
-      <c r="C6" s="124"/>
-      <c r="D6" s="124"/>
-      <c r="E6" s="124"/>
-      <c r="F6" s="124"/>
-      <c r="G6" s="124"/>
-      <c r="H6" s="124"/>
-      <c r="I6" s="124"/>
-      <c r="J6" s="124"/>
-      <c r="K6" s="124"/>
-      <c r="L6" s="124"/>
-      <c r="M6" s="124"/>
-      <c r="N6" s="125"/>
-    </row>
-    <row r="7" spans="2:14" ht="15.6">
-      <c r="B7" s="105" t="s">
+      <c r="C6" s="111"/>
+      <c r="D6" s="111"/>
+      <c r="E6" s="111"/>
+      <c r="F6" s="111"/>
+      <c r="G6" s="111"/>
+      <c r="H6" s="111"/>
+      <c r="I6" s="111"/>
+      <c r="J6" s="111"/>
+      <c r="K6" s="111"/>
+      <c r="L6" s="111"/>
+      <c r="M6" s="111"/>
+      <c r="N6" s="112"/>
+    </row>
+    <row r="7" spans="2:14" ht="15.6" x14ac:dyDescent="0.3">
+      <c r="B7" s="124" t="s">
         <v>5</v>
       </c>
-      <c r="C7" s="106"/>
-      <c r="D7" s="106"/>
-      <c r="E7" s="106"/>
-      <c r="F7" s="106"/>
-      <c r="G7" s="107"/>
-      <c r="H7" s="105" t="s">
+      <c r="C7" s="125"/>
+      <c r="D7" s="125"/>
+      <c r="E7" s="125"/>
+      <c r="F7" s="125"/>
+      <c r="G7" s="126"/>
+      <c r="H7" s="124" t="s">
         <v>6</v>
       </c>
-      <c r="I7" s="106"/>
-      <c r="J7" s="106"/>
-      <c r="K7" s="106"/>
-      <c r="L7" s="106"/>
-      <c r="M7" s="106"/>
-      <c r="N7" s="107"/>
-    </row>
-    <row r="8" spans="2:14" ht="29.25" customHeight="1">
-      <c r="B8" s="85" t="s">
+      <c r="I7" s="125"/>
+      <c r="J7" s="125"/>
+      <c r="K7" s="125"/>
+      <c r="L7" s="125"/>
+      <c r="M7" s="125"/>
+      <c r="N7" s="126"/>
+    </row>
+    <row r="8" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="122" t="s">
         <v>7</v>
       </c>
-      <c r="C8" s="86"/>
-      <c r="D8" s="45"/>
-      <c r="E8" s="113"/>
-      <c r="F8" s="113"/>
-      <c r="G8" s="46"/>
-      <c r="H8" s="80" t="s">
+      <c r="C8" s="123"/>
+      <c r="D8" s="43"/>
+      <c r="E8" s="44"/>
+      <c r="F8" s="44"/>
+      <c r="G8" s="45"/>
+      <c r="H8" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="81"/>
-      <c r="J8" s="82"/>
-      <c r="K8" s="83"/>
-      <c r="L8" s="83"/>
-      <c r="M8" s="83"/>
-      <c r="N8" s="84"/>
-    </row>
-    <row r="9" spans="2:14" ht="29.25" customHeight="1">
-      <c r="B9" s="85" t="s">
+      <c r="I8" s="27"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="119"/>
+      <c r="L8" s="120"/>
+      <c r="M8" s="120"/>
+      <c r="N8" s="121"/>
+    </row>
+    <row r="9" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="122" t="s">
         <v>8</v>
       </c>
-      <c r="C9" s="86"/>
-      <c r="D9" s="110"/>
-      <c r="E9" s="111"/>
-      <c r="F9" s="111"/>
-      <c r="G9" s="112"/>
-      <c r="H9" s="80" t="s">
+      <c r="C9" s="123"/>
+      <c r="D9" s="23"/>
+      <c r="E9" s="24"/>
+      <c r="F9" s="24"/>
+      <c r="G9" s="25"/>
+      <c r="H9" s="26" t="s">
         <v>8</v>
       </c>
-      <c r="I9" s="81"/>
-      <c r="J9" s="82"/>
-      <c r="K9" s="83"/>
-      <c r="L9" s="83"/>
-      <c r="M9" s="83"/>
-      <c r="N9" s="84"/>
-    </row>
-    <row r="10" spans="2:14" ht="29.25" customHeight="1">
-      <c r="B10" s="108" t="s">
+      <c r="I9" s="27"/>
+      <c r="J9" s="28"/>
+      <c r="K9" s="119"/>
+      <c r="L9" s="120"/>
+      <c r="M9" s="120"/>
+      <c r="N9" s="121"/>
+    </row>
+    <row r="10" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="C10" s="109"/>
-      <c r="D10" s="110"/>
-      <c r="E10" s="111"/>
-      <c r="F10" s="111"/>
-      <c r="G10" s="112"/>
-      <c r="H10" s="108" t="s">
+      <c r="C10" s="28"/>
+      <c r="D10" s="23"/>
+      <c r="E10" s="24"/>
+      <c r="F10" s="24"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="26" t="s">
         <v>9</v>
       </c>
-      <c r="I10" s="109"/>
-      <c r="J10" s="109"/>
-      <c r="K10" s="83"/>
-      <c r="L10" s="83"/>
-      <c r="M10" s="83"/>
-      <c r="N10" s="84"/>
-    </row>
-    <row r="11" spans="2:14" ht="29.25" customHeight="1">
-      <c r="B11" s="85" t="s">
+      <c r="I10" s="27"/>
+      <c r="J10" s="28"/>
+      <c r="K10" s="119"/>
+      <c r="L10" s="120"/>
+      <c r="M10" s="120"/>
+      <c r="N10" s="121"/>
+    </row>
+    <row r="11" spans="2:14" ht="29.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="122" t="s">
         <v>10</v>
       </c>
-      <c r="C11" s="86"/>
-      <c r="D11" s="110"/>
-      <c r="E11" s="111"/>
-      <c r="F11" s="111"/>
-      <c r="G11" s="112"/>
-      <c r="H11" s="108" t="s">
+      <c r="C11" s="123"/>
+      <c r="D11" s="23"/>
+      <c r="E11" s="24"/>
+      <c r="F11" s="24"/>
+      <c r="G11" s="25"/>
+      <c r="H11" s="26" t="s">
         <v>10</v>
       </c>
-      <c r="I11" s="109"/>
-      <c r="J11" s="109"/>
-      <c r="K11" s="83"/>
-      <c r="L11" s="83"/>
-      <c r="M11" s="83"/>
-      <c r="N11" s="84"/>
-    </row>
-    <row r="12" spans="2:14" ht="49.5" customHeight="1">
-      <c r="B12" s="108" t="s">
+      <c r="I11" s="27"/>
+      <c r="J11" s="28"/>
+      <c r="K11" s="119"/>
+      <c r="L11" s="120"/>
+      <c r="M11" s="120"/>
+      <c r="N11" s="121"/>
+    </row>
+    <row r="12" spans="2:14" ht="49.5" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="C12" s="109"/>
-      <c r="D12" s="110"/>
-      <c r="E12" s="111"/>
-      <c r="F12" s="111"/>
-      <c r="G12" s="112"/>
-      <c r="H12" s="108" t="s">
+      <c r="C12" s="28"/>
+      <c r="D12" s="23"/>
+      <c r="E12" s="24"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="25"/>
+      <c r="H12" s="26" t="s">
         <v>11</v>
       </c>
-      <c r="I12" s="109"/>
-      <c r="J12" s="109"/>
-      <c r="K12" s="83"/>
-      <c r="L12" s="83"/>
-      <c r="M12" s="83"/>
-      <c r="N12" s="84"/>
-    </row>
-    <row r="13" spans="2:14" s="20" customFormat="1" ht="71.400000000000006" customHeight="1">
-      <c r="B13" s="19"/>
-      <c r="C13" s="152" t="s">
+      <c r="I12" s="27"/>
+      <c r="J12" s="28"/>
+      <c r="K12" s="119"/>
+      <c r="L12" s="120"/>
+      <c r="M12" s="120"/>
+      <c r="N12" s="121"/>
+    </row>
+    <row r="13" spans="2:14" s="18" customFormat="1" ht="71.400000000000006" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B13" s="17"/>
+      <c r="C13" s="32" t="s">
         <v>44</v>
       </c>
-      <c r="D13" s="152"/>
-      <c r="E13" s="152"/>
-      <c r="F13" s="152"/>
-      <c r="G13" s="152"/>
-      <c r="H13" s="152"/>
-      <c r="I13" s="152"/>
-      <c r="J13" s="152"/>
-      <c r="K13" s="152"/>
-      <c r="L13" s="152"/>
-      <c r="M13" s="152"/>
-      <c r="N13" s="152"/>
-    </row>
-    <row r="14" spans="2:14" ht="96" customHeight="1" thickBot="1">
-      <c r="B14" s="145" t="s">
+      <c r="D13" s="32"/>
+      <c r="E13" s="32"/>
+      <c r="F13" s="32"/>
+      <c r="G13" s="32"/>
+      <c r="H13" s="32"/>
+      <c r="I13" s="32"/>
+      <c r="J13" s="32"/>
+      <c r="K13" s="32"/>
+      <c r="L13" s="32"/>
+      <c r="M13" s="32"/>
+      <c r="N13" s="32"/>
+    </row>
+    <row r="14" spans="2:14" ht="96" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B14" s="116" t="s">
         <v>12</v>
       </c>
-      <c r="C14" s="146"/>
-      <c r="D14" s="147"/>
-      <c r="E14" s="148"/>
-      <c r="F14" s="148"/>
-      <c r="G14" s="149"/>
-      <c r="H14" s="145" t="s">
+      <c r="C14" s="118"/>
+      <c r="D14" s="29"/>
+      <c r="E14" s="30"/>
+      <c r="F14" s="30"/>
+      <c r="G14" s="31"/>
+      <c r="H14" s="116" t="s">
         <v>12</v>
       </c>
-      <c r="I14" s="146"/>
-      <c r="J14" s="146"/>
-      <c r="K14" s="150"/>
-      <c r="L14" s="150"/>
-      <c r="M14" s="150"/>
-      <c r="N14" s="151"/>
-    </row>
-    <row r="15" spans="2:14" ht="15" thickBot="1">
+      <c r="I14" s="117"/>
+      <c r="J14" s="118"/>
+      <c r="K14" s="113"/>
+      <c r="L14" s="114"/>
+      <c r="M14" s="114"/>
+      <c r="N14" s="115"/>
+    </row>
+    <row r="15" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
       <c r="D15" s="8"/>
@@ -3022,351 +2965,351 @@
       <c r="M15" s="8"/>
       <c r="N15" s="8"/>
     </row>
-    <row r="16" spans="2:14" ht="21.6" thickBot="1">
-      <c r="B16" s="94" t="s">
+    <row r="16" spans="2:14" ht="21.6" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B16" s="110" t="s">
         <v>1</v>
       </c>
-      <c r="C16" s="95"/>
-      <c r="D16" s="95"/>
-      <c r="E16" s="95"/>
-      <c r="F16" s="95"/>
-      <c r="G16" s="95"/>
-      <c r="H16" s="95"/>
-      <c r="I16" s="95"/>
-      <c r="J16" s="95"/>
-      <c r="K16" s="95"/>
-      <c r="L16" s="95"/>
-      <c r="M16" s="95"/>
-      <c r="N16" s="96"/>
-    </row>
-    <row r="17" spans="2:14" ht="15.6">
-      <c r="B17" s="97" t="s">
+      <c r="C16" s="111"/>
+      <c r="D16" s="111"/>
+      <c r="E16" s="111"/>
+      <c r="F16" s="111"/>
+      <c r="G16" s="111"/>
+      <c r="H16" s="111"/>
+      <c r="I16" s="111"/>
+      <c r="J16" s="111"/>
+      <c r="K16" s="111"/>
+      <c r="L16" s="111"/>
+      <c r="M16" s="111"/>
+      <c r="N16" s="112"/>
+    </row>
+    <row r="17" spans="2:14" ht="15.6" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B17" s="107" t="s">
         <v>13</v>
       </c>
-      <c r="C17" s="98"/>
-      <c r="D17" s="98"/>
-      <c r="E17" s="98"/>
-      <c r="F17" s="98"/>
-      <c r="G17" s="98"/>
-      <c r="H17" s="98"/>
-      <c r="I17" s="99"/>
-      <c r="J17" s="100" t="s">
+      <c r="C17" s="108"/>
+      <c r="D17" s="108"/>
+      <c r="E17" s="108"/>
+      <c r="F17" s="108"/>
+      <c r="G17" s="108"/>
+      <c r="H17" s="108"/>
+      <c r="I17" s="109"/>
+      <c r="J17" s="104" t="s">
         <v>14</v>
       </c>
-      <c r="K17" s="101"/>
-      <c r="L17" s="102"/>
-      <c r="M17" s="103" t="s">
+      <c r="K17" s="105"/>
+      <c r="L17" s="106"/>
+      <c r="M17" s="102" t="s">
         <v>15</v>
       </c>
-      <c r="N17" s="104"/>
-    </row>
-    <row r="18" spans="2:14" ht="67.95" customHeight="1">
-      <c r="B18" s="140" t="s">
+      <c r="N17" s="103"/>
+    </row>
+    <row r="18" spans="2:14" ht="67.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B18" s="101" t="s">
         <v>16</v>
       </c>
-      <c r="C18" s="141"/>
-      <c r="D18" s="142"/>
-      <c r="E18" s="142"/>
-      <c r="F18" s="141" t="s">
+      <c r="C18" s="98"/>
+      <c r="D18" s="99"/>
+      <c r="E18" s="100"/>
+      <c r="F18" s="38" t="s">
         <v>17</v>
       </c>
-      <c r="G18" s="141"/>
-      <c r="H18" s="67"/>
-      <c r="I18" s="68"/>
-      <c r="J18" s="143" t="s">
+      <c r="G18" s="98"/>
+      <c r="H18" s="96"/>
+      <c r="I18" s="97"/>
+      <c r="J18" s="94" t="s">
         <v>35</v>
       </c>
-      <c r="K18" s="144"/>
-      <c r="L18" s="22"/>
-      <c r="M18" s="126" t="s">
+      <c r="K18" s="95"/>
+      <c r="L18" s="20"/>
+      <c r="M18" s="92" t="s">
         <v>39</v>
       </c>
-      <c r="N18" s="129" t="s">
+      <c r="N18" s="33" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="19" spans="2:14" ht="23.25" customHeight="1">
-      <c r="B19" s="132" t="s">
+    <row r="19" spans="2:14" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="83" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="133"/>
-      <c r="D19" s="135" t="s">
+      <c r="C19" s="36"/>
+      <c r="D19" s="89" t="s">
         <v>20</v>
       </c>
-      <c r="E19" s="135"/>
-      <c r="F19" s="135"/>
-      <c r="G19" s="135"/>
-      <c r="H19" s="135"/>
-      <c r="I19" s="136"/>
-      <c r="J19" s="137" t="s">
+      <c r="E19" s="90"/>
+      <c r="F19" s="90"/>
+      <c r="G19" s="90"/>
+      <c r="H19" s="90"/>
+      <c r="I19" s="91"/>
+      <c r="J19" s="86" t="s">
         <v>21</v>
       </c>
-      <c r="K19" s="138"/>
-      <c r="L19" s="139"/>
-      <c r="M19" s="127"/>
-      <c r="N19" s="130"/>
-    </row>
-    <row r="20" spans="2:14" ht="31.95" customHeight="1">
-      <c r="B20" s="134"/>
-      <c r="C20" s="133"/>
-      <c r="D20" s="10" t="s">
+      <c r="K19" s="87"/>
+      <c r="L19" s="88"/>
+      <c r="M19" s="93"/>
+      <c r="N19" s="34"/>
+    </row>
+    <row r="20" spans="2:14" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="36"/>
+      <c r="C20" s="36"/>
+      <c r="D20" s="22" t="s">
         <v>22</v>
       </c>
-      <c r="E20" s="10" t="s">
+      <c r="E20" s="22" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="10" t="s">
+      <c r="F20" s="22" t="s">
         <v>38</v>
       </c>
-      <c r="G20" s="10" t="s">
+      <c r="G20" s="22" t="s">
         <v>24</v>
       </c>
-      <c r="H20" s="10" t="s">
+      <c r="H20" s="22" t="s">
         <v>25</v>
       </c>
-      <c r="I20" s="11" t="s">
+      <c r="I20" s="22" t="s">
         <v>26</v>
       </c>
-      <c r="J20" s="137" t="s">
+      <c r="J20" s="37" t="s">
         <v>27</v>
       </c>
-      <c r="K20" s="138"/>
-      <c r="L20" s="139"/>
-      <c r="M20" s="128"/>
-      <c r="N20" s="131"/>
-    </row>
-    <row r="21" spans="2:14" ht="51" customHeight="1">
-      <c r="B21" s="23"/>
-      <c r="C21" s="24"/>
-      <c r="D21" s="24"/>
-      <c r="E21" s="25"/>
-      <c r="F21" s="26"/>
-      <c r="G21" s="24"/>
-      <c r="H21" s="27"/>
-      <c r="I21" s="28"/>
-      <c r="J21" s="29"/>
-      <c r="K21" s="45"/>
-      <c r="L21" s="46"/>
-      <c r="M21" s="30"/>
-      <c r="N21" s="31"/>
-    </row>
-    <row r="22" spans="2:14" ht="51" customHeight="1">
-      <c r="B22" s="32"/>
-      <c r="C22" s="25"/>
-      <c r="D22" s="25"/>
-      <c r="E22" s="25"/>
-      <c r="F22" s="33"/>
-      <c r="G22" s="25"/>
-      <c r="H22" s="27"/>
-      <c r="I22" s="28"/>
-      <c r="J22" s="29"/>
-      <c r="K22" s="45"/>
-      <c r="L22" s="46"/>
-      <c r="M22" s="34"/>
-      <c r="N22" s="35"/>
-    </row>
-    <row r="23" spans="2:14" ht="51" customHeight="1">
-      <c r="B23" s="23"/>
-      <c r="C23" s="24"/>
-      <c r="D23" s="24"/>
-      <c r="E23" s="25"/>
-      <c r="F23" s="26"/>
-      <c r="G23" s="24"/>
-      <c r="H23" s="27"/>
-      <c r="I23" s="28"/>
-      <c r="J23" s="29"/>
-      <c r="K23" s="45"/>
-      <c r="L23" s="46"/>
-      <c r="M23" s="30"/>
-      <c r="N23" s="31"/>
-    </row>
-    <row r="24" spans="2:14" ht="51" customHeight="1">
-      <c r="B24" s="32"/>
-      <c r="C24" s="25"/>
-      <c r="D24" s="25"/>
-      <c r="E24" s="25"/>
-      <c r="F24" s="33"/>
-      <c r="G24" s="25"/>
-      <c r="H24" s="27"/>
-      <c r="I24" s="28"/>
-      <c r="J24" s="29"/>
-      <c r="K24" s="45"/>
-      <c r="L24" s="46"/>
-      <c r="M24" s="34"/>
-      <c r="N24" s="35"/>
-    </row>
-    <row r="25" spans="2:14" ht="51" customHeight="1">
-      <c r="B25" s="32"/>
-      <c r="C25" s="25"/>
-      <c r="D25" s="25"/>
-      <c r="E25" s="25"/>
-      <c r="F25" s="33"/>
-      <c r="G25" s="25"/>
-      <c r="H25" s="27"/>
-      <c r="I25" s="28"/>
-      <c r="J25" s="29"/>
-      <c r="K25" s="45"/>
-      <c r="L25" s="46"/>
-      <c r="M25" s="34"/>
-      <c r="N25" s="35"/>
-    </row>
-    <row r="26" spans="2:14" ht="51" customHeight="1">
-      <c r="B26" s="32"/>
-      <c r="C26" s="25"/>
-      <c r="D26" s="25"/>
-      <c r="E26" s="25"/>
-      <c r="F26" s="33"/>
-      <c r="G26" s="25"/>
-      <c r="H26" s="27"/>
-      <c r="I26" s="28"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="45"/>
-      <c r="L26" s="46"/>
-      <c r="M26" s="34"/>
-      <c r="N26" s="35"/>
-    </row>
-    <row r="27" spans="2:14" ht="51" customHeight="1">
-      <c r="B27" s="32"/>
-      <c r="C27" s="25"/>
-      <c r="D27" s="25"/>
-      <c r="E27" s="25"/>
-      <c r="F27" s="33"/>
-      <c r="G27" s="25"/>
-      <c r="H27" s="27"/>
-      <c r="I27" s="28"/>
-      <c r="J27" s="29"/>
-      <c r="K27" s="45"/>
-      <c r="L27" s="46"/>
-      <c r="M27" s="34"/>
-      <c r="N27" s="35"/>
-    </row>
-    <row r="28" spans="2:14" ht="51" customHeight="1">
-      <c r="B28" s="32"/>
-      <c r="C28" s="25"/>
-      <c r="D28" s="25"/>
-      <c r="E28" s="25"/>
-      <c r="F28" s="33"/>
-      <c r="G28" s="25"/>
-      <c r="H28" s="27"/>
-      <c r="I28" s="28"/>
-      <c r="J28" s="29"/>
-      <c r="K28" s="45"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="34"/>
-      <c r="N28" s="35"/>
-    </row>
-    <row r="29" spans="2:14" ht="51" customHeight="1">
-      <c r="B29" s="32"/>
-      <c r="C29" s="25"/>
-      <c r="D29" s="25"/>
-      <c r="E29" s="25"/>
-      <c r="F29" s="33"/>
-      <c r="G29" s="25"/>
-      <c r="H29" s="27"/>
-      <c r="I29" s="28"/>
-      <c r="J29" s="29"/>
-      <c r="K29" s="45"/>
-      <c r="L29" s="46"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="35"/>
-    </row>
-    <row r="30" spans="2:14" ht="51" customHeight="1">
-      <c r="B30" s="23"/>
-      <c r="C30" s="24"/>
-      <c r="D30" s="24"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="26"/>
-      <c r="G30" s="24"/>
-      <c r="H30" s="27"/>
-      <c r="I30" s="28"/>
-      <c r="J30" s="29"/>
-      <c r="K30" s="45"/>
-      <c r="L30" s="46"/>
-      <c r="M30" s="30"/>
-      <c r="N30" s="31"/>
-    </row>
-    <row r="31" spans="2:14" ht="51" customHeight="1">
-      <c r="B31" s="32"/>
-      <c r="C31" s="25"/>
-      <c r="D31" s="25"/>
-      <c r="E31" s="25"/>
-      <c r="F31" s="33"/>
-      <c r="G31" s="25"/>
-      <c r="H31" s="27"/>
-      <c r="I31" s="28"/>
-      <c r="J31" s="29"/>
-      <c r="K31" s="45"/>
-      <c r="L31" s="46"/>
-      <c r="M31" s="34"/>
-      <c r="N31" s="35"/>
-    </row>
-    <row r="32" spans="2:14" ht="51" customHeight="1">
-      <c r="B32" s="23"/>
-      <c r="C32" s="24"/>
-      <c r="D32" s="24"/>
-      <c r="E32" s="25"/>
-      <c r="F32" s="26"/>
-      <c r="G32" s="24"/>
-      <c r="H32" s="27"/>
-      <c r="I32" s="28"/>
-      <c r="J32" s="29"/>
-      <c r="K32" s="45"/>
-      <c r="L32" s="46"/>
-      <c r="M32" s="30"/>
-      <c r="N32" s="31"/>
-    </row>
-    <row r="33" spans="2:14" ht="51" customHeight="1">
-      <c r="B33" s="32"/>
-      <c r="C33" s="25"/>
-      <c r="D33" s="25"/>
-      <c r="E33" s="25"/>
-      <c r="F33" s="33"/>
-      <c r="G33" s="25"/>
-      <c r="H33" s="27"/>
-      <c r="I33" s="28"/>
-      <c r="J33" s="29"/>
-      <c r="K33" s="45"/>
-      <c r="L33" s="46"/>
-      <c r="M33" s="34"/>
-      <c r="N33" s="35"/>
-    </row>
-    <row r="34" spans="2:14" ht="51" customHeight="1">
-      <c r="B34" s="23"/>
-      <c r="C34" s="24"/>
-      <c r="D34" s="24"/>
-      <c r="E34" s="25"/>
-      <c r="F34" s="26"/>
-      <c r="G34" s="24"/>
-      <c r="H34" s="27"/>
-      <c r="I34" s="28"/>
-      <c r="J34" s="29"/>
-      <c r="K34" s="45"/>
-      <c r="L34" s="46"/>
-      <c r="M34" s="30"/>
-      <c r="N34" s="31"/>
-    </row>
-    <row r="35" spans="2:14" ht="51" customHeight="1" thickBot="1">
-      <c r="B35" s="36"/>
-      <c r="C35" s="37"/>
-      <c r="D35" s="37"/>
-      <c r="E35" s="37"/>
-      <c r="F35" s="40"/>
-      <c r="G35" s="37"/>
-      <c r="H35" s="41"/>
-      <c r="I35" s="42"/>
-      <c r="J35" s="43"/>
-      <c r="K35" s="92"/>
-      <c r="L35" s="93"/>
-      <c r="M35" s="38"/>
-      <c r="N35" s="44"/>
-    </row>
-    <row r="36" spans="2:14" ht="23.4">
-      <c r="B36" s="12"/>
-      <c r="C36" s="13"/>
-      <c r="D36" s="13"/>
-      <c r="E36" s="13"/>
-      <c r="F36" s="39"/>
-      <c r="G36" s="14"/>
+      <c r="K20" s="37"/>
+      <c r="L20" s="85"/>
+      <c r="M20" s="84"/>
+      <c r="N20" s="35"/>
+    </row>
+    <row r="21" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B21" s="135"/>
+      <c r="C21" s="136"/>
+      <c r="D21" s="136"/>
+      <c r="E21" s="137"/>
+      <c r="F21" s="82"/>
+      <c r="G21" s="136"/>
+      <c r="H21" s="138"/>
+      <c r="I21" s="139"/>
+      <c r="J21" s="139"/>
+      <c r="K21" s="140"/>
+      <c r="L21" s="140"/>
+      <c r="M21" s="141"/>
+      <c r="N21" s="142"/>
+    </row>
+    <row r="22" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B22" s="144"/>
+      <c r="C22" s="137"/>
+      <c r="D22" s="137"/>
+      <c r="E22" s="137"/>
+      <c r="F22" s="145"/>
+      <c r="G22" s="137"/>
+      <c r="H22" s="138"/>
+      <c r="I22" s="139"/>
+      <c r="J22" s="139"/>
+      <c r="K22" s="140"/>
+      <c r="L22" s="140"/>
+      <c r="M22" s="146"/>
+      <c r="N22" s="147"/>
+    </row>
+    <row r="23" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B23" s="135"/>
+      <c r="C23" s="136"/>
+      <c r="D23" s="136"/>
+      <c r="E23" s="137"/>
+      <c r="F23" s="82"/>
+      <c r="G23" s="136"/>
+      <c r="H23" s="138"/>
+      <c r="I23" s="139"/>
+      <c r="J23" s="139"/>
+      <c r="K23" s="140"/>
+      <c r="L23" s="140"/>
+      <c r="M23" s="141"/>
+      <c r="N23" s="142"/>
+    </row>
+    <row r="24" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B24" s="144"/>
+      <c r="C24" s="137"/>
+      <c r="D24" s="137"/>
+      <c r="E24" s="137"/>
+      <c r="F24" s="145"/>
+      <c r="G24" s="137"/>
+      <c r="H24" s="138"/>
+      <c r="I24" s="139"/>
+      <c r="J24" s="139"/>
+      <c r="K24" s="140"/>
+      <c r="L24" s="140"/>
+      <c r="M24" s="146"/>
+      <c r="N24" s="147"/>
+    </row>
+    <row r="25" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B25" s="144"/>
+      <c r="C25" s="137"/>
+      <c r="D25" s="137"/>
+      <c r="E25" s="137"/>
+      <c r="F25" s="145"/>
+      <c r="G25" s="137"/>
+      <c r="H25" s="138"/>
+      <c r="I25" s="139"/>
+      <c r="J25" s="139"/>
+      <c r="K25" s="140"/>
+      <c r="L25" s="140"/>
+      <c r="M25" s="146"/>
+      <c r="N25" s="147"/>
+    </row>
+    <row r="26" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="144"/>
+      <c r="C26" s="137"/>
+      <c r="D26" s="137"/>
+      <c r="E26" s="137"/>
+      <c r="F26" s="145"/>
+      <c r="G26" s="137"/>
+      <c r="H26" s="138"/>
+      <c r="I26" s="139"/>
+      <c r="J26" s="139"/>
+      <c r="K26" s="140"/>
+      <c r="L26" s="140"/>
+      <c r="M26" s="146"/>
+      <c r="N26" s="147"/>
+    </row>
+    <row r="27" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B27" s="144"/>
+      <c r="C27" s="137"/>
+      <c r="D27" s="137"/>
+      <c r="E27" s="137"/>
+      <c r="F27" s="145"/>
+      <c r="G27" s="137"/>
+      <c r="H27" s="138"/>
+      <c r="I27" s="139"/>
+      <c r="J27" s="139"/>
+      <c r="K27" s="140"/>
+      <c r="L27" s="140"/>
+      <c r="M27" s="146"/>
+      <c r="N27" s="147"/>
+    </row>
+    <row r="28" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B28" s="144"/>
+      <c r="C28" s="137"/>
+      <c r="D28" s="137"/>
+      <c r="E28" s="137"/>
+      <c r="F28" s="145"/>
+      <c r="G28" s="137"/>
+      <c r="H28" s="138"/>
+      <c r="I28" s="139"/>
+      <c r="J28" s="139"/>
+      <c r="K28" s="140"/>
+      <c r="L28" s="140"/>
+      <c r="M28" s="146"/>
+      <c r="N28" s="147"/>
+    </row>
+    <row r="29" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B29" s="144"/>
+      <c r="C29" s="137"/>
+      <c r="D29" s="137"/>
+      <c r="E29" s="137"/>
+      <c r="F29" s="145"/>
+      <c r="G29" s="137"/>
+      <c r="H29" s="138"/>
+      <c r="I29" s="139"/>
+      <c r="J29" s="139"/>
+      <c r="K29" s="140"/>
+      <c r="L29" s="140"/>
+      <c r="M29" s="146"/>
+      <c r="N29" s="147"/>
+    </row>
+    <row r="30" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B30" s="135"/>
+      <c r="C30" s="136"/>
+      <c r="D30" s="136"/>
+      <c r="E30" s="137"/>
+      <c r="F30" s="82"/>
+      <c r="G30" s="136"/>
+      <c r="H30" s="138"/>
+      <c r="I30" s="139"/>
+      <c r="J30" s="139"/>
+      <c r="K30" s="140"/>
+      <c r="L30" s="140"/>
+      <c r="M30" s="141"/>
+      <c r="N30" s="142"/>
+    </row>
+    <row r="31" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B31" s="144"/>
+      <c r="C31" s="137"/>
+      <c r="D31" s="137"/>
+      <c r="E31" s="137"/>
+      <c r="F31" s="145"/>
+      <c r="G31" s="137"/>
+      <c r="H31" s="138"/>
+      <c r="I31" s="139"/>
+      <c r="J31" s="139"/>
+      <c r="K31" s="140"/>
+      <c r="L31" s="140"/>
+      <c r="M31" s="146"/>
+      <c r="N31" s="147"/>
+    </row>
+    <row r="32" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B32" s="135"/>
+      <c r="C32" s="136"/>
+      <c r="D32" s="136"/>
+      <c r="E32" s="137"/>
+      <c r="F32" s="82"/>
+      <c r="G32" s="136"/>
+      <c r="H32" s="138"/>
+      <c r="I32" s="139"/>
+      <c r="J32" s="139"/>
+      <c r="K32" s="140"/>
+      <c r="L32" s="140"/>
+      <c r="M32" s="141"/>
+      <c r="N32" s="142"/>
+    </row>
+    <row r="33" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="144"/>
+      <c r="C33" s="137"/>
+      <c r="D33" s="137"/>
+      <c r="E33" s="137"/>
+      <c r="F33" s="145"/>
+      <c r="G33" s="137"/>
+      <c r="H33" s="138"/>
+      <c r="I33" s="139"/>
+      <c r="J33" s="139"/>
+      <c r="K33" s="140"/>
+      <c r="L33" s="140"/>
+      <c r="M33" s="146"/>
+      <c r="N33" s="147"/>
+    </row>
+    <row r="34" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B34" s="135"/>
+      <c r="C34" s="136"/>
+      <c r="D34" s="136"/>
+      <c r="E34" s="137"/>
+      <c r="F34" s="82"/>
+      <c r="G34" s="136"/>
+      <c r="H34" s="138"/>
+      <c r="I34" s="139"/>
+      <c r="J34" s="139"/>
+      <c r="K34" s="140"/>
+      <c r="L34" s="140"/>
+      <c r="M34" s="141"/>
+      <c r="N34" s="142"/>
+    </row>
+    <row r="35" spans="2:14" s="143" customFormat="1" ht="51" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="144"/>
+      <c r="C35" s="137"/>
+      <c r="D35" s="137"/>
+      <c r="E35" s="137"/>
+      <c r="F35" s="145"/>
+      <c r="G35" s="137"/>
+      <c r="H35" s="138"/>
+      <c r="I35" s="139"/>
+      <c r="J35" s="139"/>
+      <c r="K35" s="140"/>
+      <c r="L35" s="140"/>
+      <c r="M35" s="146"/>
+      <c r="N35" s="147"/>
+    </row>
+    <row r="36" spans="2:14" ht="23.4" x14ac:dyDescent="0.3">
+      <c r="B36" s="10"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="12"/>
       <c r="H36" s="6"/>
       <c r="I36" s="6"/>
       <c r="J36" s="7"/>
@@ -3375,13 +3318,13 @@
       <c r="M36" s="1"/>
       <c r="N36" s="1"/>
     </row>
-    <row r="37" spans="2:14" ht="15" thickBot="1">
-      <c r="B37" s="15"/>
-      <c r="C37" s="13"/>
-      <c r="D37" s="13"/>
-      <c r="E37" s="13"/>
+    <row r="37" spans="2:14" ht="15" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B37" s="13"/>
+      <c r="C37" s="11"/>
+      <c r="D37" s="11"/>
+      <c r="E37" s="11"/>
       <c r="F37" s="1"/>
-      <c r="G37" s="16"/>
+      <c r="G37" s="14"/>
       <c r="H37" s="6"/>
       <c r="I37" s="6"/>
       <c r="J37" s="7"/>
@@ -3390,174 +3333,192 @@
       <c r="M37" s="6"/>
       <c r="N37" s="6"/>
     </row>
-    <row r="38" spans="2:14" ht="75" customHeight="1">
-      <c r="B38" s="87" t="s">
+    <row r="38" spans="2:14" ht="75" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B38" s="51" t="s">
         <v>42</v>
       </c>
-      <c r="C38" s="88"/>
-      <c r="D38" s="89" t="s">
+      <c r="C38" s="52"/>
+      <c r="D38" s="53" t="s">
         <v>2</v>
       </c>
-      <c r="E38" s="90"/>
-      <c r="F38" s="90"/>
-      <c r="G38" s="90"/>
-      <c r="H38" s="90"/>
-      <c r="I38" s="90"/>
-      <c r="J38" s="90"/>
-      <c r="K38" s="90"/>
-      <c r="L38" s="90"/>
-      <c r="M38" s="90"/>
-      <c r="N38" s="91"/>
-    </row>
-    <row r="39" spans="2:14" ht="58.95" customHeight="1">
-      <c r="B39" s="52" t="s">
+      <c r="E38" s="54"/>
+      <c r="F38" s="54"/>
+      <c r="G38" s="54"/>
+      <c r="H38" s="54"/>
+      <c r="I38" s="54"/>
+      <c r="J38" s="54"/>
+      <c r="K38" s="54"/>
+      <c r="L38" s="54"/>
+      <c r="M38" s="54"/>
+      <c r="N38" s="55"/>
+    </row>
+    <row r="39" spans="2:14" ht="58.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="C39" s="53"/>
-      <c r="D39" s="54" t="s">
+      <c r="C39" s="62"/>
+      <c r="D39" s="63" t="s">
         <v>28</v>
       </c>
-      <c r="E39" s="55"/>
-      <c r="F39" s="55"/>
-      <c r="G39" s="55" t="s">
+      <c r="E39" s="64"/>
+      <c r="F39" s="64"/>
+      <c r="G39" s="64" t="s">
         <v>29</v>
       </c>
-      <c r="H39" s="55"/>
-      <c r="I39" s="55" t="s">
+      <c r="H39" s="64"/>
+      <c r="I39" s="64" t="s">
         <v>30</v>
       </c>
-      <c r="J39" s="55"/>
-      <c r="K39" s="55"/>
-      <c r="L39" s="55"/>
-      <c r="M39" s="56" t="s">
+      <c r="J39" s="64"/>
+      <c r="K39" s="64"/>
+      <c r="L39" s="64"/>
+      <c r="M39" s="65" t="s">
         <v>31</v>
       </c>
-      <c r="N39" s="57"/>
-    </row>
-    <row r="40" spans="2:14" ht="48" customHeight="1">
-      <c r="B40" s="58"/>
-      <c r="C40" s="59"/>
-      <c r="D40" s="60"/>
-      <c r="E40" s="61"/>
-      <c r="F40" s="61"/>
-      <c r="G40" s="64"/>
-      <c r="H40" s="64"/>
-      <c r="I40" s="18" t="s">
+      <c r="N39" s="66"/>
+    </row>
+    <row r="40" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="67"/>
+      <c r="C40" s="68"/>
+      <c r="D40" s="69"/>
+      <c r="E40" s="70"/>
+      <c r="F40" s="70"/>
+      <c r="G40" s="73"/>
+      <c r="H40" s="73"/>
+      <c r="I40" s="16" t="s">
         <v>36</v>
       </c>
-      <c r="J40" s="66"/>
-      <c r="K40" s="66"/>
-      <c r="L40" s="66"/>
-      <c r="M40" s="67"/>
-      <c r="N40" s="68"/>
-    </row>
-    <row r="41" spans="2:14" ht="48" customHeight="1">
-      <c r="B41" s="52" t="s">
+      <c r="J40" s="75"/>
+      <c r="K40" s="75"/>
+      <c r="L40" s="75"/>
+      <c r="M40" s="39"/>
+      <c r="N40" s="40"/>
+    </row>
+    <row r="41" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B41" s="61" t="s">
         <v>40</v>
       </c>
-      <c r="C41" s="71"/>
-      <c r="D41" s="60"/>
-      <c r="E41" s="61"/>
-      <c r="F41" s="61"/>
-      <c r="G41" s="64"/>
-      <c r="H41" s="64"/>
-      <c r="I41" s="72" t="s">
+      <c r="C41" s="78"/>
+      <c r="D41" s="69"/>
+      <c r="E41" s="70"/>
+      <c r="F41" s="70"/>
+      <c r="G41" s="73"/>
+      <c r="H41" s="73"/>
+      <c r="I41" s="79" t="s">
         <v>37</v>
       </c>
-      <c r="J41" s="66"/>
-      <c r="K41" s="66"/>
-      <c r="L41" s="66"/>
-      <c r="M41" s="67"/>
-      <c r="N41" s="68"/>
-    </row>
-    <row r="42" spans="2:14" ht="48" customHeight="1" thickBot="1">
-      <c r="B42" s="75"/>
-      <c r="C42" s="76"/>
-      <c r="D42" s="62"/>
-      <c r="E42" s="63"/>
-      <c r="F42" s="63"/>
-      <c r="G42" s="65"/>
-      <c r="H42" s="65"/>
-      <c r="I42" s="73"/>
-      <c r="J42" s="74"/>
-      <c r="K42" s="74"/>
-      <c r="L42" s="74"/>
-      <c r="M42" s="69"/>
-      <c r="N42" s="70"/>
-    </row>
-    <row r="43" spans="2:14" ht="48" customHeight="1">
-      <c r="B43" s="77" t="s">
+      <c r="J41" s="75"/>
+      <c r="K41" s="75"/>
+      <c r="L41" s="75"/>
+      <c r="M41" s="39"/>
+      <c r="N41" s="40"/>
+    </row>
+    <row r="42" spans="2:14" ht="48" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B42" s="46"/>
+      <c r="C42" s="47"/>
+      <c r="D42" s="71"/>
+      <c r="E42" s="72"/>
+      <c r="F42" s="72"/>
+      <c r="G42" s="74"/>
+      <c r="H42" s="74"/>
+      <c r="I42" s="80"/>
+      <c r="J42" s="81"/>
+      <c r="K42" s="81"/>
+      <c r="L42" s="81"/>
+      <c r="M42" s="76"/>
+      <c r="N42" s="77"/>
+    </row>
+    <row r="43" spans="2:14" ht="48" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B43" s="48" t="s">
         <v>32</v>
       </c>
-      <c r="C43" s="78"/>
-      <c r="D43" s="78"/>
-      <c r="E43" s="78"/>
-      <c r="F43" s="78"/>
-      <c r="G43" s="78"/>
-      <c r="H43" s="78"/>
-      <c r="I43" s="78"/>
-      <c r="J43" s="78"/>
-      <c r="K43" s="78"/>
-      <c r="L43" s="78"/>
-      <c r="M43" s="78"/>
-      <c r="N43" s="79"/>
-    </row>
-    <row r="44" spans="2:14" ht="104.25" customHeight="1" thickBot="1">
-      <c r="B44" s="47" t="s">
+      <c r="C43" s="49"/>
+      <c r="D43" s="49"/>
+      <c r="E43" s="49"/>
+      <c r="F43" s="49"/>
+      <c r="G43" s="49"/>
+      <c r="H43" s="49"/>
+      <c r="I43" s="49"/>
+      <c r="J43" s="49"/>
+      <c r="K43" s="49"/>
+      <c r="L43" s="49"/>
+      <c r="M43" s="49"/>
+      <c r="N43" s="50"/>
+    </row>
+    <row r="44" spans="2:14" ht="104.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="B44" s="56" t="s">
         <v>33</v>
       </c>
-      <c r="C44" s="48"/>
-      <c r="D44" s="49"/>
-      <c r="E44" s="49"/>
-      <c r="F44" s="49"/>
-      <c r="G44" s="49"/>
-      <c r="H44" s="49"/>
-      <c r="I44" s="17" t="s">
+      <c r="C44" s="57"/>
+      <c r="D44" s="58"/>
+      <c r="E44" s="58"/>
+      <c r="F44" s="58"/>
+      <c r="G44" s="58"/>
+      <c r="H44" s="58"/>
+      <c r="I44" s="15" t="s">
         <v>34</v>
       </c>
-      <c r="J44" s="50"/>
-      <c r="K44" s="50"/>
-      <c r="L44" s="50"/>
-      <c r="M44" s="50"/>
-      <c r="N44" s="51"/>
-    </row>
-    <row r="46" spans="2:14">
-      <c r="B46" s="21" t="s">
+      <c r="J44" s="59"/>
+      <c r="K44" s="59"/>
+      <c r="L44" s="59"/>
+      <c r="M44" s="59"/>
+      <c r="N44" s="60"/>
+    </row>
+    <row r="46" spans="2:14" x14ac:dyDescent="0.3">
+      <c r="B46" s="19" t="s">
         <v>43</v>
       </c>
-      <c r="C46" s="21"/>
-      <c r="D46" s="21"/>
-      <c r="E46" s="21"/>
-      <c r="F46" s="21"/>
-      <c r="G46" s="21"/>
+      <c r="C46" s="19"/>
+      <c r="D46" s="19"/>
+      <c r="E46" s="19"/>
+      <c r="F46" s="19"/>
+      <c r="G46" s="19"/>
     </row>
   </sheetData>
-  <sheetProtection algorithmName="SHA-512" hashValue="x/6J+a6KNWyGCeyRKKn5FHJlrEY4NiA1OcA0xmMANbmYzYqFnapIYVF+nNvbD3yr5Y8LEVqf1hgPxEiAZXacig==" saltValue="jHtw/EV+dCMB27kTi1VNHg==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1"/>
   <mergeCells count="82">
-    <mergeCell ref="D9:G9"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="K9:N9"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="D14:G14"/>
-    <mergeCell ref="H14:J14"/>
-    <mergeCell ref="K14:N14"/>
-    <mergeCell ref="C13:N13"/>
-    <mergeCell ref="M18:M20"/>
-    <mergeCell ref="N18:N20"/>
-    <mergeCell ref="B19:C20"/>
-    <mergeCell ref="D19:I19"/>
-    <mergeCell ref="J19:L19"/>
-    <mergeCell ref="J20:L20"/>
-    <mergeCell ref="B18:C18"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="F18:G18"/>
-    <mergeCell ref="H18:I18"/>
-    <mergeCell ref="J18:K18"/>
-    <mergeCell ref="B2:L2"/>
-    <mergeCell ref="M2:N2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:N4"/>
-    <mergeCell ref="B6:N6"/>
+    <mergeCell ref="K8:N8"/>
+    <mergeCell ref="H8:J8"/>
+    <mergeCell ref="M17:N17"/>
+    <mergeCell ref="J17:L17"/>
+    <mergeCell ref="B17:I17"/>
+    <mergeCell ref="B16:N16"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="K35:L35"/>
+    <mergeCell ref="K24:L24"/>
+    <mergeCell ref="K23:L23"/>
+    <mergeCell ref="K22:L22"/>
+    <mergeCell ref="K21:L21"/>
+    <mergeCell ref="K30:L30"/>
+    <mergeCell ref="K31:L31"/>
+    <mergeCell ref="K32:L32"/>
+    <mergeCell ref="K33:L33"/>
+    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="K25:L25"/>
+    <mergeCell ref="K26:L26"/>
+    <mergeCell ref="K27:L27"/>
+    <mergeCell ref="K28:L28"/>
+    <mergeCell ref="K29:L29"/>
+    <mergeCell ref="B44:C44"/>
+    <mergeCell ref="D44:H44"/>
+    <mergeCell ref="J44:N44"/>
+    <mergeCell ref="B39:C39"/>
+    <mergeCell ref="D39:F39"/>
+    <mergeCell ref="G39:H39"/>
+    <mergeCell ref="I39:L39"/>
+    <mergeCell ref="M39:N39"/>
+    <mergeCell ref="B40:C40"/>
+    <mergeCell ref="D40:F42"/>
+    <mergeCell ref="G40:H42"/>
+    <mergeCell ref="J40:L40"/>
+    <mergeCell ref="M40:N42"/>
+    <mergeCell ref="B41:C41"/>
+    <mergeCell ref="I41:I42"/>
+    <mergeCell ref="J41:L42"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B43:N43"/>
+    <mergeCell ref="B38:C38"/>
+    <mergeCell ref="D38:N38"/>
     <mergeCell ref="B7:G7"/>
     <mergeCell ref="H7:N7"/>
     <mergeCell ref="B12:C12"/>
@@ -3574,48 +3535,30 @@
     <mergeCell ref="K11:N11"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="D8:G8"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B43:N43"/>
-    <mergeCell ref="H8:J8"/>
-    <mergeCell ref="K8:N8"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="B38:C38"/>
-    <mergeCell ref="D38:N38"/>
-    <mergeCell ref="K21:L21"/>
-    <mergeCell ref="K22:L22"/>
-    <mergeCell ref="K23:L23"/>
-    <mergeCell ref="K24:L24"/>
-    <mergeCell ref="K35:L35"/>
-    <mergeCell ref="B16:N16"/>
-    <mergeCell ref="B17:I17"/>
-    <mergeCell ref="J17:L17"/>
-    <mergeCell ref="M17:N17"/>
-    <mergeCell ref="B44:C44"/>
-    <mergeCell ref="D44:H44"/>
-    <mergeCell ref="J44:N44"/>
-    <mergeCell ref="B39:C39"/>
-    <mergeCell ref="D39:F39"/>
-    <mergeCell ref="G39:H39"/>
-    <mergeCell ref="I39:L39"/>
-    <mergeCell ref="M39:N39"/>
-    <mergeCell ref="B40:C40"/>
-    <mergeCell ref="D40:F42"/>
-    <mergeCell ref="G40:H42"/>
-    <mergeCell ref="J40:L40"/>
-    <mergeCell ref="M40:N42"/>
-    <mergeCell ref="B41:C41"/>
-    <mergeCell ref="I41:I42"/>
-    <mergeCell ref="J41:L42"/>
-    <mergeCell ref="K25:L25"/>
-    <mergeCell ref="K26:L26"/>
-    <mergeCell ref="K27:L27"/>
-    <mergeCell ref="K28:L28"/>
-    <mergeCell ref="K29:L29"/>
-    <mergeCell ref="K30:L30"/>
-    <mergeCell ref="K31:L31"/>
-    <mergeCell ref="K32:L32"/>
-    <mergeCell ref="K33:L33"/>
-    <mergeCell ref="K34:L34"/>
+    <mergeCell ref="B2:L2"/>
+    <mergeCell ref="M2:N2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:N4"/>
+    <mergeCell ref="B6:N6"/>
+    <mergeCell ref="M18:M20"/>
+    <mergeCell ref="N18:N20"/>
+    <mergeCell ref="B19:C20"/>
+    <mergeCell ref="D19:I19"/>
+    <mergeCell ref="J19:L19"/>
+    <mergeCell ref="J20:L20"/>
+    <mergeCell ref="B18:C18"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="F18:G18"/>
+    <mergeCell ref="H18:I18"/>
+    <mergeCell ref="J18:K18"/>
+    <mergeCell ref="D9:G9"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="K9:N9"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="D14:G14"/>
+    <mergeCell ref="H14:J14"/>
+    <mergeCell ref="K14:N14"/>
+    <mergeCell ref="C13:N13"/>
   </mergeCells>
   <conditionalFormatting sqref="B40:C40">
     <cfRule type="cellIs" dxfId="3" priority="1" operator="equal">
@@ -3639,7 +3582,7 @@
     <hyperlink ref="B46" r:id="rId1" display="La versión descargable del formato se encuentra disponible en el Portafolio de la Gestión del Rendimiento."/>
   </hyperlinks>
   <pageMargins left="0.25" right="0.25" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="40" orientation="portrait" r:id="rId2"/>
+  <pageSetup paperSize="9" scale="37" orientation="portrait" r:id="rId2"/>
   <drawing r:id="rId3"/>
   <legacyDrawing r:id="rId4"/>
 </worksheet>

</xml_diff>